<commit_message>
prepara archivos excel para simulacion final
</commit_message>
<xml_diff>
--- a/Resultados/Entregable/Reporte_Dip_SinInc_vf_2.xlsx
+++ b/Resultados/Entregable/Reporte_Dip_SinInc_vf_2.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ivan\Desktop\Ivan\Laboral\EstrategiaSur\GitProjects\Proyeccion-electoral-congreso\Resultados\Entregable\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CA2527A-7708-4F4C-83FA-F0546B042E5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D7BF4FE-FD3A-4ACA-9080-8A0573319064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1665" windowWidth="29040" windowHeight="15720" activeTab="15" xr2:uid="{85AAF8D7-1A96-46DE-A921-B4694576F524}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{85AAF8D7-1A96-46DE-A921-B4694576F524}"/>
   </bookViews>
   <sheets>
-    <sheet name="Resumen de Pactos" sheetId="32" r:id="rId1"/>
+    <sheet name="Resumen de Pactos" sheetId="33" r:id="rId1"/>
     <sheet name="D3" sheetId="1" r:id="rId2"/>
     <sheet name="D5" sheetId="16" r:id="rId3"/>
     <sheet name="D6" sheetId="17" r:id="rId4"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="776" uniqueCount="78">
   <si>
     <t>Esc</t>
   </si>
@@ -733,6 +733,12 @@
       <t>- Para observar el modelo con el factor de incumbencias revisar el archivo "Reporte_Dip.xlsx"</t>
     </r>
   </si>
+  <si>
+    <t>Personalizado 3 CHV+</t>
+  </si>
+  <si>
+    <t>Personalizado 3 CHV</t>
+  </si>
 </sst>
 </file>
 
@@ -1072,7 +1078,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1146,12 +1152,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="115">
+  <dxfs count="142">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1169,13 +1190,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FF7030A0"/>
         </patternFill>
       </fill>
@@ -1183,7 +1197,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF00B050"/>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1197,21 +1211,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFABAB"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1249,7 +1249,21 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="-0.499984740745262"/>
+          <bgColor rgb="FFFFABAB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1263,7 +1277,171 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFABAB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1292,6 +1470,128 @@
       <fill>
         <patternFill>
           <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFABAB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1333,20 +1633,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor theme="2" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
@@ -1354,45 +1640,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFABAB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
+          <bgColor rgb="FF7030A0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1406,7 +1654,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF7030A0"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1434,7 +1689,45 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFABAB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1469,13 +1762,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FF0070C0"/>
         </patternFill>
       </fill>
@@ -1484,107 +1770,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFABAB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0070C0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1640,14 +1825,21 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFFF00"/>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1678,14 +1870,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
+          <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1699,6 +1884,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="2" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
@@ -1706,14 +1898,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF7030A0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1727,21 +1912,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0070C0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1762,6 +1933,20 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="5" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
@@ -1769,7 +1954,21 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1797,13 +1996,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FFFFABAB"/>
         </patternFill>
       </fill>
@@ -1815,6 +2007,20 @@
       <fill>
         <patternFill>
           <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1856,13 +2062,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
@@ -1871,6 +2070,13 @@
       <fill>
         <patternFill>
           <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1919,7 +2125,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1933,14 +2146,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="-0.499984740745262"/>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
+          <bgColor theme="5" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1954,21 +2167,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF0070C0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2004,14 +2203,14 @@
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>13599</xdr:rowOff>
+      <xdr:rowOff>7249</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Imagen 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{062922E4-BF1D-43D1-8169-2A772A608603}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4F47A803-6E75-43E1-AE14-44C9D6D90B30}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2033,8 +2232,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="809626" y="5868213"/>
-          <a:ext cx="4448174" cy="555711"/>
+          <a:off x="809626" y="5950763"/>
+          <a:ext cx="4448174" cy="558886"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2058,10 +2257,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Imagen 8">
+        <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A2A312F9-2DFE-40C0-B00A-B4F5669007D2}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7D946038-6C76-4833-81A6-2C8210E3435F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2083,8 +2282,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6819901" y="5868213"/>
-          <a:ext cx="4444999" cy="549361"/>
+          <a:off x="6819901" y="5950763"/>
+          <a:ext cx="4444999" cy="558886"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2108,10 +2307,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="Imagen 10">
+        <xdr:cNvPr id="4" name="Imagen 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{46900199-EB6E-4126-93A8-D3513A9A9345}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{698CF99D-4D7A-45D0-B2F6-A4DEECDEB91E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2133,8 +2332,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12836526" y="5868213"/>
-          <a:ext cx="4448174" cy="552536"/>
+          <a:off x="12836526" y="5950763"/>
+          <a:ext cx="4448174" cy="562061"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2158,10 +2357,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="Imagen 11">
+        <xdr:cNvPr id="5" name="Imagen 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{93D81DFD-0E7F-4D90-9B60-60F8C01063BC}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B014BCF2-F5FE-4777-A316-87C6381C2C39}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2183,8 +2382,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="18865851" y="5868213"/>
-          <a:ext cx="4448174" cy="552536"/>
+          <a:off x="18865851" y="5950763"/>
+          <a:ext cx="4448174" cy="562061"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2208,10 +2407,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="13" name="Imagen 12">
+        <xdr:cNvPr id="6" name="Imagen 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1DCB3C95-6A37-49A7-864D-A037785005A8}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{64D8508E-9F08-4EFD-84B8-AE199B579A45}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2233,8 +2432,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="24888826" y="5868213"/>
-          <a:ext cx="4448174" cy="549361"/>
+          <a:off x="24888826" y="5950763"/>
+          <a:ext cx="4448174" cy="558886"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2258,10 +2457,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="14" name="Imagen 13">
+        <xdr:cNvPr id="7" name="Imagen 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{35C7F400-C14A-4A8B-8AD2-433E72E90580}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EE6EB0EB-6A93-4550-A57E-D05FCD20D072}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2283,8 +2482,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="30914976" y="5868213"/>
-          <a:ext cx="4441824" cy="552536"/>
+          <a:off x="30914976" y="5950763"/>
+          <a:ext cx="4441824" cy="562061"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2308,10 +2507,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="15" name="Imagen 14">
+        <xdr:cNvPr id="8" name="Imagen 7">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{022A9296-BA67-4B28-99E4-FC87F4DC2375}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8F683600-3FBE-4DC4-9038-2A74F31B6254}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2333,8 +2532,108 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="36928426" y="5868213"/>
-          <a:ext cx="4448174" cy="552536"/>
+          <a:off x="36928426" y="5950763"/>
+          <a:ext cx="4448174" cy="562061"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>19051</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>172263</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>3438525</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>181874</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Imagen 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{488AB0F0-F865-4CDE-81E2-606E5B6851F6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="42919651" y="5938063"/>
+          <a:ext cx="4448174" cy="562061"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>33</xdr:col>
+      <xdr:colOff>6351</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>172263</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>3425825</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>181874</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Imagen 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{34BA2377-1F1E-4E2B-874C-5384AFF34085}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="48926751" y="5938063"/>
+          <a:ext cx="4448174" cy="562061"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -24868,8 +25167,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90F7F12D-1B3C-4B35-ABFD-7D1C6B7F9B07}">
-  <dimension ref="B2:AA27"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32D65D37-C3FD-4538-9692-FE05F9C4D931}">
+  <dimension ref="B2:AI27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="14.7265625" customWidth="1"/>
@@ -24886,9 +25185,13 @@
     <col min="23" max="23" width="49.6328125" customWidth="1"/>
     <col min="26" max="26" width="14.7265625" customWidth="1"/>
     <col min="27" max="27" width="49.6328125" customWidth="1"/>
+    <col min="30" max="30" width="14.7265625" customWidth="1"/>
+    <col min="31" max="31" width="49.6328125" customWidth="1"/>
+    <col min="34" max="34" width="14.7265625" customWidth="1"/>
+    <col min="35" max="35" width="49.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
@@ -24931,8 +25234,20 @@
       <c r="AA2" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="AD2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="AE2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="AH2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI2" s="2" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="3" spans="2:27" ht="77" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:35" ht="77" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="10" t="s">
         <v>8</v>
       </c>
@@ -24987,8 +25302,20 @@
       <c r="AA3" s="31" t="s">
         <v>36</v>
       </c>
+      <c r="AD3" s="31" t="s">
+        <v>76</v>
+      </c>
+      <c r="AE3" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="AH3" s="31" t="s">
+        <v>77</v>
+      </c>
+      <c r="AI3" s="31" t="s">
+        <v>36</v>
+      </c>
     </row>
-    <row r="4" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B4" s="33" t="s">
         <v>40</v>
       </c>
@@ -25043,8 +25370,20 @@
       <c r="AA4" s="33" t="s">
         <v>41</v>
       </c>
+      <c r="AD4" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="AE4" s="33" t="s">
+        <v>41</v>
+      </c>
+      <c r="AH4" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="AI4" s="33" t="s">
+        <v>41</v>
+      </c>
     </row>
-    <row r="5" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B5" s="11" t="s">
         <v>11</v>
       </c>
@@ -25087,8 +25426,20 @@
       <c r="AA5" s="12" t="s">
         <v>42</v>
       </c>
+      <c r="AD5" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="AE5" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH5" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="AI5" s="12" t="s">
+        <v>42</v>
+      </c>
     </row>
-    <row r="6" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B6" s="11" t="s">
         <v>12</v>
       </c>
@@ -25131,8 +25482,20 @@
       <c r="AA6" s="12" t="s">
         <v>42</v>
       </c>
+      <c r="AD6" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE6" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH6" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="AI6" s="12" t="s">
+        <v>42</v>
+      </c>
     </row>
-    <row r="7" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B7" s="11" t="s">
         <v>38</v>
       </c>
@@ -25175,8 +25538,20 @@
       <c r="AA7" s="12" t="s">
         <v>42</v>
       </c>
+      <c r="AD7" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="AE7" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH7" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="AI7" s="12" t="s">
+        <v>42</v>
+      </c>
     </row>
-    <row r="8" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B8" s="11" t="s">
         <v>17</v>
       </c>
@@ -25219,8 +25594,20 @@
       <c r="AA8" s="12" t="s">
         <v>42</v>
       </c>
+      <c r="AD8" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE8" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH8" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI8" s="12" t="s">
+        <v>42</v>
+      </c>
     </row>
-    <row r="9" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B9" s="13" t="s">
         <v>23</v>
       </c>
@@ -25263,8 +25650,20 @@
       <c r="AA9" s="12" t="s">
         <v>42</v>
       </c>
+      <c r="AD9" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="AE9" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH9" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="AI9" s="12" t="s">
+        <v>42</v>
+      </c>
     </row>
-    <row r="10" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B10" s="13" t="s">
         <v>13</v>
       </c>
@@ -25307,8 +25706,20 @@
       <c r="AA10" s="12" t="s">
         <v>43</v>
       </c>
+      <c r="AD10" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="AE10" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH10" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="AI10" s="12" t="s">
+        <v>42</v>
+      </c>
     </row>
-    <row r="11" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B11" s="13" t="s">
         <v>19</v>
       </c>
@@ -25351,8 +25762,20 @@
       <c r="AA11" s="12" t="s">
         <v>43</v>
       </c>
+      <c r="AD11" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="AE11" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH11" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="AI11" s="12" t="s">
+        <v>42</v>
+      </c>
     </row>
-    <row r="12" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B12" s="13" t="s">
         <v>15</v>
       </c>
@@ -25395,8 +25818,20 @@
       <c r="AA12" s="12" t="s">
         <v>43</v>
       </c>
+      <c r="AD12" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE12" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH12" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI12" s="12" t="s">
+        <v>42</v>
+      </c>
     </row>
-    <row r="13" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B13" s="13" t="s">
         <v>26</v>
       </c>
@@ -25439,8 +25874,20 @@
       <c r="AA13" s="12" t="s">
         <v>43</v>
       </c>
+      <c r="AD13" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="AE13" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH13" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="AI13" s="12" t="s">
+        <v>42</v>
+      </c>
     </row>
-    <row r="14" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B14" s="14" t="s">
         <v>21</v>
       </c>
@@ -25483,8 +25930,20 @@
       <c r="AA14" s="12" t="s">
         <v>44</v>
       </c>
+      <c r="AD14" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="AE14" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="AH14" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="AI14" s="20" t="s">
+        <v>43</v>
+      </c>
     </row>
-    <row r="15" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B15" s="14" t="s">
         <v>24</v>
       </c>
@@ -25527,8 +25986,20 @@
       <c r="AA15" s="12" t="s">
         <v>44</v>
       </c>
+      <c r="AD15" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="AE15" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="AH15" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="AI15" s="12" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="16" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B16" s="14" t="s">
         <v>16</v>
       </c>
@@ -25571,8 +26042,20 @@
       <c r="AA16" s="12" t="s">
         <v>44</v>
       </c>
+      <c r="AD16" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="AE16" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="AH16" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="AI16" s="12" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="17" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B17" s="14" t="s">
         <v>27</v>
       </c>
@@ -25615,8 +26098,20 @@
       <c r="AA17" s="12" t="s">
         <v>46</v>
       </c>
+      <c r="AD17" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="AE17" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="AH17" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="AI17" s="12" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="18" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B18" s="14" t="s">
         <v>20</v>
       </c>
@@ -25659,8 +26154,20 @@
       <c r="AA18" s="12" t="s">
         <v>46</v>
       </c>
+      <c r="AD18" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="AE18" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="AH18" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="AI18" s="12" t="s">
+        <v>46</v>
+      </c>
     </row>
-    <row r="19" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B19" s="14" t="s">
         <v>14</v>
       </c>
@@ -25703,8 +26210,20 @@
       <c r="AA19" s="12" t="s">
         <v>47</v>
       </c>
+      <c r="AD19" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="AE19" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="AH19" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="AI19" s="12" t="s">
+        <v>46</v>
+      </c>
     </row>
-    <row r="20" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B20" s="14" t="s">
         <v>22</v>
       </c>
@@ -25747,8 +26266,20 @@
       <c r="AA20" s="12" t="s">
         <v>47</v>
       </c>
+      <c r="AD20" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="AE20" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="AH20" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="AI20" s="12" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="21" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B21" s="15" t="s">
         <v>45</v>
       </c>
@@ -25791,8 +26322,20 @@
       <c r="AA21" s="12" t="s">
         <v>47</v>
       </c>
+      <c r="AD21" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE21" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="AH21" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="AI21" s="12" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="22" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B22" s="16" t="s">
         <v>18</v>
       </c>
@@ -25835,8 +26378,20 @@
       <c r="AA22" s="12" t="s">
         <v>47</v>
       </c>
+      <c r="AD22" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="AE22" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="AH22" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="AI22" s="12" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="23" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B23" s="17" t="s">
         <v>25</v>
       </c>
@@ -25879,8 +26434,20 @@
       <c r="AA23" s="12" t="s">
         <v>48</v>
       </c>
+      <c r="AD23" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="AE23" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="AH23" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="AI23" s="12" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="24" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B24" s="18" t="s">
         <v>49</v>
       </c>
@@ -25923,8 +26490,20 @@
       <c r="AA24" s="12" t="s">
         <v>48</v>
       </c>
+      <c r="AD24" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="AE24" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="AH24" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="AI24" s="12" t="s">
+        <v>48</v>
+      </c>
     </row>
-    <row r="25" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B25" s="18" t="s">
         <v>39</v>
       </c>
@@ -25967,8 +26546,20 @@
       <c r="AA25" s="12" t="s">
         <v>50</v>
       </c>
+      <c r="AD25" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="AE25" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="AH25" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="AI25" s="12" t="s">
+        <v>48</v>
+      </c>
     </row>
-    <row r="26" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B26" s="18" t="s">
         <v>51</v>
       </c>
@@ -26011,8 +26602,20 @@
       <c r="AA26" s="12" t="s">
         <v>52</v>
       </c>
+      <c r="AD26" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="AE26" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="AH26" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="AI26" s="12" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="27" spans="2:27" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:35" x14ac:dyDescent="0.35">
       <c r="B27" s="19" t="s">
         <v>37</v>
       </c>
@@ -26054,388 +26657,489 @@
       </c>
       <c r="AA27" s="20" t="s">
         <v>53</v>
+      </c>
+      <c r="AD27" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="AE27" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="AH27" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="AI27" s="12" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B4:C27">
-    <cfRule type="cellIs" dxfId="114" priority="120" operator="equal">
+    <cfRule type="cellIs" dxfId="140" priority="136" operator="equal">
+      <formula>"p7"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="138" priority="137" operator="equal">
+      <formula>"p6"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="139" priority="138" operator="equal">
+      <formula>"p5"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="137" priority="139" operator="equal">
+      <formula>"p4"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="136" priority="140" operator="equal">
       <formula>"p3"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="113" priority="122" operator="equal">
-      <formula>"p1"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="112" priority="121" operator="equal">
+    <cfRule type="cellIs" dxfId="135" priority="141" operator="equal">
       <formula>"p2"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="111" priority="116" operator="equal">
-      <formula>"p7"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="110" priority="117" operator="equal">
-      <formula>"p6"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="109" priority="118" operator="equal">
-      <formula>"p5"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="108" priority="119" operator="equal">
-      <formula>"p4"</formula>
+    <cfRule type="cellIs" dxfId="141" priority="142" operator="equal">
+      <formula>"p1"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F4:G27">
-    <cfRule type="cellIs" dxfId="107" priority="73" operator="equal">
-      <formula>"p1"</formula>
+    <cfRule type="cellIs" dxfId="130" priority="94" operator="equal">
+      <formula>"p7"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="106" priority="71" operator="equal">
+    <cfRule type="cellIs" dxfId="131" priority="95" operator="equal">
+      <formula>"p6"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="132" priority="96" operator="equal">
+      <formula>"p5"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="133" priority="97" operator="equal">
+      <formula>"p4"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="134" priority="98" operator="equal">
       <formula>"p3"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="105" priority="70" operator="equal">
-      <formula>"p4"</formula>
+    <cfRule type="cellIs" dxfId="129" priority="99" operator="equal">
+      <formula>"p2"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="104" priority="69" operator="equal">
-      <formula>"p5"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="103" priority="68" operator="equal">
-      <formula>"p6"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="102" priority="67" operator="equal">
-      <formula>"p7"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="101" priority="72" operator="equal">
-      <formula>"p2"</formula>
+    <cfRule type="cellIs" dxfId="128" priority="100" operator="equal">
+      <formula>"p1"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F5:G27">
-    <cfRule type="cellIs" dxfId="100" priority="66" operator="equal">
+    <cfRule type="cellIs" dxfId="127" priority="93" operator="equal">
       <formula>"p8"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J4:K4">
-    <cfRule type="cellIs" dxfId="99" priority="102" operator="equal">
+    <cfRule type="cellIs" dxfId="126" priority="129" operator="equal">
       <formula>"p7"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="98" priority="104" operator="equal">
+    <cfRule type="cellIs" dxfId="125" priority="130" operator="equal">
+      <formula>"p6"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="120" priority="131" operator="equal">
       <formula>"p5"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="97" priority="103" operator="equal">
-      <formula>"p6"</formula>
+    <cfRule type="cellIs" dxfId="121" priority="132" operator="equal">
+      <formula>"p4"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="96" priority="108" operator="equal">
+    <cfRule type="cellIs" dxfId="122" priority="133" operator="equal">
+      <formula>"p3"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="123" priority="134" operator="equal">
+      <formula>"p2"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="124" priority="135" operator="equal">
       <formula>"p1"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="95" priority="107" operator="equal">
-      <formula>"p2"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="94" priority="106" operator="equal">
-      <formula>"p3"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="93" priority="105" operator="equal">
-      <formula>"p4"</formula>
-    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J5:K27">
-    <cfRule type="cellIs" dxfId="92" priority="53" operator="equal">
+  <conditionalFormatting sqref="J5:K27 AD5:AE27">
+    <cfRule type="cellIs" dxfId="118" priority="80" operator="equal">
       <formula>"p13"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="91" priority="54" operator="equal">
+    <cfRule type="cellIs" dxfId="117" priority="81" operator="equal">
       <formula>"p12"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="90" priority="55" operator="equal">
+    <cfRule type="cellIs" dxfId="119" priority="82" operator="equal">
       <formula>"p11"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="89" priority="56" operator="equal">
+    <cfRule type="cellIs" dxfId="116" priority="83" operator="equal">
       <formula>"p10"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="88" priority="57" operator="equal">
+    <cfRule type="cellIs" dxfId="115" priority="84" operator="equal">
       <formula>"p9"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:K27">
-    <cfRule type="cellIs" dxfId="87" priority="65" operator="equal">
-      <formula>"p1"</formula>
+  <conditionalFormatting sqref="K5:K27 AE5:AE27">
+    <cfRule type="cellIs" dxfId="107" priority="85" operator="equal">
+      <formula>"p8"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="86" priority="60" operator="equal">
+    <cfRule type="cellIs" dxfId="108" priority="86" operator="equal">
+      <formula>"p7"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="109" priority="87" operator="equal">
       <formula>"p6"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="85" priority="61" operator="equal">
+    <cfRule type="cellIs" dxfId="110" priority="88" operator="equal">
       <formula>"p5"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="84" priority="58" operator="equal">
-      <formula>"p8"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="83" priority="62" operator="equal">
+    <cfRule type="cellIs" dxfId="113" priority="89" operator="equal">
       <formula>"p4"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="82" priority="63" operator="equal">
+    <cfRule type="cellIs" dxfId="111" priority="90" operator="equal">
       <formula>"p3"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="81" priority="64" operator="equal">
+    <cfRule type="cellIs" dxfId="112" priority="91" operator="equal">
       <formula>"p2"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="80" priority="59" operator="equal">
-      <formula>"p7"</formula>
+    <cfRule type="cellIs" dxfId="114" priority="92" operator="equal">
+      <formula>"p1"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N4:O4">
-    <cfRule type="cellIs" dxfId="79" priority="100" operator="equal">
+    <cfRule type="cellIs" dxfId="101" priority="122" operator="equal">
+      <formula>"p7"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="102" priority="123" operator="equal">
+      <formula>"p6"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="100" priority="124" operator="equal">
+      <formula>"p5"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="106" priority="125" operator="equal">
+      <formula>"p4"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="103" priority="126" operator="equal">
+      <formula>"p3"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="104" priority="127" operator="equal">
       <formula>"p2"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="78" priority="101" operator="equal">
+    <cfRule type="cellIs" dxfId="105" priority="128" operator="equal">
       <formula>"p1"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="77" priority="95" operator="equal">
-      <formula>"p7"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="76" priority="96" operator="equal">
-      <formula>"p6"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="75" priority="97" operator="equal">
-      <formula>"p5"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="74" priority="98" operator="equal">
-      <formula>"p4"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="73" priority="99" operator="equal">
-      <formula>"p3"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N5:O27">
-    <cfRule type="cellIs" dxfId="72" priority="42" operator="equal">
+    <cfRule type="cellIs" dxfId="96" priority="67" operator="equal">
+      <formula>"p13"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="97" priority="68" operator="equal">
+      <formula>"p12"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="98" priority="69" operator="equal">
       <formula>"p11"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="71" priority="41" operator="equal">
-      <formula>"p12"</formula>
+    <cfRule type="cellIs" dxfId="95" priority="70" operator="equal">
+      <formula>"p10"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="70" priority="40" operator="equal">
-      <formula>"p13"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="69" priority="44" operator="equal">
+    <cfRule type="cellIs" dxfId="99" priority="71" operator="equal">
       <formula>"p9"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="68" priority="43" operator="equal">
-      <formula>"p10"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O5:O27">
-    <cfRule type="cellIs" dxfId="67" priority="47" operator="equal">
+    <cfRule type="cellIs" dxfId="94" priority="72" operator="equal">
+      <formula>"p8"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="93" priority="73" operator="equal">
+      <formula>"p7"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="92" priority="74" operator="equal">
       <formula>"p6"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="66" priority="48" operator="equal">
+    <cfRule type="cellIs" dxfId="91" priority="75" operator="equal">
       <formula>"p5"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="65" priority="49" operator="equal">
+    <cfRule type="cellIs" dxfId="90" priority="76" operator="equal">
       <formula>"p4"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="64" priority="50" operator="equal">
+    <cfRule type="cellIs" dxfId="89" priority="77" operator="equal">
       <formula>"p3"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="63" priority="51" operator="equal">
+    <cfRule type="cellIs" dxfId="88" priority="78" operator="equal">
       <formula>"p2"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="62" priority="52" operator="equal">
+    <cfRule type="cellIs" dxfId="87" priority="79" operator="equal">
       <formula>"p1"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="61" priority="46" operator="equal">
-      <formula>"p7"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="45" operator="equal">
-      <formula>"p8"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R4:S4">
-    <cfRule type="cellIs" dxfId="59" priority="90" operator="equal">
+    <cfRule type="cellIs" dxfId="86" priority="115" operator="equal">
+      <formula>"p7"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="80" priority="116" operator="equal">
+      <formula>"p6"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="81" priority="117" operator="equal">
       <formula>"p5"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="89" operator="equal">
-      <formula>"p6"</formula>
+    <cfRule type="cellIs" dxfId="82" priority="118" operator="equal">
+      <formula>"p4"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="57" priority="93" operator="equal">
+    <cfRule type="cellIs" dxfId="83" priority="119" operator="equal">
+      <formula>"p3"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="84" priority="120" operator="equal">
       <formula>"p2"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="92" operator="equal">
-      <formula>"p3"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="55" priority="88" operator="equal">
-      <formula>"p7"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="91" operator="equal">
-      <formula>"p4"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="53" priority="94" operator="equal">
+    <cfRule type="cellIs" dxfId="85" priority="121" operator="equal">
       <formula>"p1"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R5:S27">
-    <cfRule type="cellIs" dxfId="52" priority="29" operator="equal">
+    <cfRule type="cellIs" dxfId="75" priority="54" operator="equal">
+      <formula>"p13"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="78" priority="55" operator="equal">
+      <formula>"p12"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="76" priority="56" operator="equal">
       <formula>"p11"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="27" operator="equal">
-      <formula>"p13"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="28" operator="equal">
-      <formula>"p12"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="30" operator="equal">
+    <cfRule type="cellIs" dxfId="77" priority="57" operator="equal">
       <formula>"p10"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="31" operator="equal">
+    <cfRule type="cellIs" dxfId="79" priority="58" operator="equal">
       <formula>"p9"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S5:S27">
-    <cfRule type="cellIs" dxfId="47" priority="33" operator="equal">
+    <cfRule type="cellIs" dxfId="70" priority="59" operator="equal">
+      <formula>"p8"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="71" priority="60" operator="equal">
       <formula>"p7"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="39" operator="equal">
-      <formula>"p1"</formula>
+    <cfRule type="cellIs" dxfId="72" priority="61" operator="equal">
+      <formula>"p6"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="38" operator="equal">
+    <cfRule type="cellIs" dxfId="73" priority="62" operator="equal">
+      <formula>"p5"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="74" priority="63" operator="equal">
+      <formula>"p4"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="67" priority="64" operator="equal">
+      <formula>"p3"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="68" priority="65" operator="equal">
       <formula>"p2"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="32" operator="equal">
-      <formula>"p8"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="37" operator="equal">
-      <formula>"p3"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="36" operator="equal">
-      <formula>"p4"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="41" priority="35" operator="equal">
-      <formula>"p5"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="34" operator="equal">
-      <formula>"p6"</formula>
+    <cfRule type="cellIs" dxfId="69" priority="66" operator="equal">
+      <formula>"p1"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V4:W4">
-    <cfRule type="cellIs" dxfId="39" priority="87" operator="equal">
-      <formula>"p1"</formula>
+    <cfRule type="cellIs" dxfId="60" priority="108" operator="equal">
+      <formula>"p7"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="83" operator="equal">
+    <cfRule type="cellIs" dxfId="66" priority="109" operator="equal">
+      <formula>"p6"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="61" priority="110" operator="equal">
       <formula>"p5"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="82" operator="equal">
-      <formula>"p6"</formula>
+    <cfRule type="cellIs" dxfId="62" priority="111" operator="equal">
+      <formula>"p4"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="81" operator="equal">
-      <formula>"p7"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="35" priority="85" operator="equal">
+    <cfRule type="cellIs" dxfId="63" priority="112" operator="equal">
       <formula>"p3"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="86" operator="equal">
+    <cfRule type="cellIs" dxfId="64" priority="113" operator="equal">
       <formula>"p2"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="84" operator="equal">
-      <formula>"p4"</formula>
+    <cfRule type="cellIs" dxfId="65" priority="114" operator="equal">
+      <formula>"p1"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V5:W27">
-    <cfRule type="cellIs" dxfId="32" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="59" priority="41" operator="equal">
+      <formula>"p13"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="55" priority="42" operator="equal">
       <formula>"p12"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="56" priority="43" operator="equal">
+      <formula>"p11"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="58" priority="44" operator="equal">
       <formula>"p10"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="57" priority="45" operator="equal">
       <formula>"p9"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="29" priority="14" operator="equal">
-      <formula>"p13"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="16" operator="equal">
-      <formula>"p11"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W5:W27">
-    <cfRule type="cellIs" dxfId="27" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="54" priority="46" operator="equal">
+      <formula>"p8"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="53" priority="47" operator="equal">
+      <formula>"p7"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="52" priority="48" operator="equal">
       <formula>"p6"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="19" operator="equal">
-      <formula>"p8"</formula>
+    <cfRule type="cellIs" dxfId="51" priority="49" operator="equal">
+      <formula>"p5"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="20" operator="equal">
-      <formula>"p7"</formula>
+    <cfRule type="cellIs" dxfId="50" priority="50" operator="equal">
+      <formula>"p4"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="26" operator="equal">
-      <formula>"p1"</formula>
+    <cfRule type="cellIs" dxfId="49" priority="51" operator="equal">
+      <formula>"p3"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="23" priority="25" operator="equal">
+    <cfRule type="cellIs" dxfId="47" priority="52" operator="equal">
       <formula>"p2"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="24" operator="equal">
-      <formula>"p3"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="23" operator="equal">
-      <formula>"p4"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="22" operator="equal">
-      <formula>"p5"</formula>
+    <cfRule type="cellIs" dxfId="48" priority="53" operator="equal">
+      <formula>"p1"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z4:AA4">
-    <cfRule type="cellIs" dxfId="19" priority="77" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="101" operator="equal">
+      <formula>"p7"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="45" priority="102" operator="equal">
+      <formula>"p6"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="46" priority="103" operator="equal">
+      <formula>"p5"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="43" priority="104" operator="equal">
       <formula>"p4"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="78" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="105" operator="equal">
       <formula>"p3"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="79" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="106" operator="equal">
       <formula>"p2"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="80" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="107" operator="equal">
       <formula>"p1"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="74" operator="equal">
-      <formula>"p7"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="75" operator="equal">
-      <formula>"p6"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="76" operator="equal">
-      <formula>"p5"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z5:AA27">
-    <cfRule type="cellIs" dxfId="12" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="28" operator="equal">
+      <formula>"p13"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="38" priority="29" operator="equal">
+      <formula>"p12"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="37" priority="30" operator="equal">
       <formula>"p11"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="31" operator="equal">
       <formula>"p10"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="32" operator="equal">
       <formula>"p9"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
-      <formula>"p13"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="2" operator="equal">
-      <formula>"p12"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA5:AA27">
+    <cfRule type="cellIs" dxfId="28" priority="33" operator="equal">
+      <formula>"p8"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="29" priority="34" operator="equal">
+      <formula>"p7"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="34" priority="35" operator="equal">
+      <formula>"p6"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="30" priority="36" operator="equal">
+      <formula>"p5"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="27" priority="37" operator="equal">
+      <formula>"p4"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="31" priority="38" operator="equal">
+      <formula>"p3"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="32" priority="39" operator="equal">
+      <formula>"p2"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="33" priority="40" operator="equal">
+      <formula>"p1"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD4:AE4">
+    <cfRule type="cellIs" dxfId="22" priority="21" operator="equal">
+      <formula>"p7"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="23" priority="22" operator="equal">
+      <formula>"p6"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="24" priority="23" operator="equal">
+      <formula>"p5"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="25" priority="24" operator="equal">
+      <formula>"p4"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="26" priority="25" operator="equal">
+      <formula>"p3"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="20" priority="26" operator="equal">
+      <formula>"p2"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="21" priority="27" operator="equal">
+      <formula>"p1"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AH4:AI4">
+    <cfRule type="cellIs" dxfId="13" priority="14" operator="equal">
+      <formula>"p7"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="15" priority="15" operator="equal">
+      <formula>"p6"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="17" priority="16" operator="equal">
+      <formula>"p5"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="18" priority="17" operator="equal">
+      <formula>"p4"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="16" priority="18" operator="equal">
+      <formula>"p3"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="19" priority="19" operator="equal">
+      <formula>"p2"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="14" priority="20" operator="equal">
+      <formula>"p1"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AH5:AI27">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+      <formula>"p13"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="2" operator="equal">
+      <formula>"p12"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="11" priority="3" operator="equal">
+      <formula>"p11"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="4" operator="equal">
+      <formula>"p10"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="5" operator="equal">
+      <formula>"p9"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI5:AI27">
     <cfRule type="cellIs" dxfId="7" priority="6" operator="equal">
       <formula>"p8"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="7" operator="equal">
       <formula>"p7"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="8" operator="equal">
       <formula>"p6"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="9" operator="equal">
+      <formula>"p5"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="10" operator="equal">
       <formula>"p4"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="11" operator="equal">
       <formula>"p3"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="9" operator="equal">
-      <formula>"p5"</formula>
+    <cfRule type="cellIs" dxfId="2" priority="12" operator="equal">
+      <formula>"p2"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="13" operator="equal">
       <formula>"p1"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="12" operator="equal">
-      <formula>"p2"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>